<commit_message>
feat(data): TMDB 인기 영화 수집·적재 import_movies 커맨드
</commit_message>
<xml_diff>
--- a/docs/04_schedule.xlsx
+++ b/docs/04_schedule.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="166">
   <si>
     <r>
       <rPr>
@@ -2169,6 +2169,98 @@
   </si>
   <si>
     <t xml:space="preserve">추천 챗봇</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.5</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">알림 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">친구 요청</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수락 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· Signal)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">알림 모델</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(F-NTF-01)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">6.1</t>
@@ -4563,7 +4655,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA33"/>
+  <dimension ref="A1:AA34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -5936,34 +6028,34 @@
       <c r="Z27" s="19"/>
       <c r="AA27" s="12"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
         <v>122</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="C28" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D28" s="18" t="s">
-        <v>115</v>
+      <c r="D28" s="14" t="s">
+        <v>40</v>
       </c>
       <c r="E28" s="6" t="n">
         <f aca="false">G28-F28+1</f>
         <v>2</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>125</v>
+        <v>13</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>98</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>37</v>
@@ -5983,20 +6075,20 @@
       <c r="U28" s="12"/>
       <c r="V28" s="12"/>
       <c r="W28" s="12"/>
-      <c r="X28" s="12"/>
-      <c r="Y28" s="12"/>
-      <c r="Z28" s="19"/>
-      <c r="AA28" s="19"/>
+      <c r="X28" s="15"/>
+      <c r="Y28" s="15"/>
+      <c r="Z28" s="12"/>
+      <c r="AA28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C29" s="8" t="s">
         <v>127</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>128</v>
       </c>
       <c r="D29" s="18" t="s">
         <v>115</v>
@@ -6011,8 +6103,8 @@
       <c r="G29" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="H29" s="6" t="s">
-        <v>122</v>
+      <c r="H29" s="7" t="s">
+        <v>128</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>129</v>
@@ -6045,9 +6137,9 @@
         <v>130</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="C30" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>131</v>
       </c>
       <c r="D30" s="18" t="s">
@@ -6055,16 +6147,16 @@
       </c>
       <c r="E30" s="6" t="n">
         <f aca="false">G30-F30+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G30" s="6" t="n">
         <v>15</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>132</v>
@@ -6089,38 +6181,90 @@
       <c r="W30" s="12"/>
       <c r="X30" s="12"/>
       <c r="Y30" s="12"/>
-      <c r="Z30" s="12"/>
+      <c r="Z30" s="19"/>
       <c r="AA30" s="19"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="Q32" s="21" t="s">
+      <c r="B31" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C31" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="V32" s="21" t="s">
+      <c r="D31" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <f aca="false">G31-F31+1</f>
+        <v>1</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="I31" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="Y32" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="AA32" s="21" t="s">
-        <v>137</v>
-      </c>
+      <c r="J31" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="13"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
+      <c r="O31" s="12"/>
+      <c r="P31" s="12"/>
+      <c r="Q31" s="12"/>
+      <c r="R31" s="12"/>
+      <c r="S31" s="12"/>
+      <c r="T31" s="12"/>
+      <c r="U31" s="12"/>
+      <c r="V31" s="12"/>
+      <c r="W31" s="12"/>
+      <c r="X31" s="12"/>
+      <c r="Y31" s="12"/>
+      <c r="Z31" s="12"/>
+      <c r="AA31" s="19"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q33" s="22" t="s">
+      <c r="A33" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q33" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="V33" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="V33" s="22" t="s">
+      <c r="Y33" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="Y33" s="22" t="s">
+      <c r="AA33" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="AA33" s="22" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q34" s="22" t="s">
         <v>141</v>
+      </c>
+      <c r="V34" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="Y34" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="AA34" s="22" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -6129,7 +6273,7 @@
     <mergeCell ref="R2:V2"/>
     <mergeCell ref="W2:AA2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J4:J30">
+  <conditionalFormatting sqref="J4:J31">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"완료"</formula>
     </cfRule>
@@ -6141,7 +6285,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J4:J30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J4:J31" type="list">
       <formula1>"할 일,진행중,완료,보류"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6171,7 +6315,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6179,43 +6323,43 @@
         <v>7</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -6242,7 +6386,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6250,7 +6394,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6258,17 +6402,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6276,17 +6420,17 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6294,7 +6438,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>